<commit_message>
1) Impute Arg, Descriptivos (7), Correls(AgB, covs), AgB's cointegrados? 2) Agregue mas covs en las correls
</commit_message>
<xml_diff>
--- a/USA/datos.xlsx
+++ b/USA/datos.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:T127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,69 +367,94 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Crude oil, Brent</t>
+          <t>Petroleo Brent</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Crude oil, WTI</t>
+          <t>Petroleo WTI</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Natural gas, US</t>
+          <t>Gas Natural EEUU</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Natural gas, Europe</t>
+          <t>Gas Natural Europa</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Soybeans</t>
+          <t>Soja</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Maize</t>
+          <t>Maiz</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Sorghum</t>
+          <t>Sorgo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Wheat, US SRW</t>
+          <t>Trigo SRW</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Wheat, US HRW</t>
+          <t>Trigo HRW</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Beef **</t>
+          <t>Carne</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Chicken **</t>
+          <t>Pollo</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>DAP</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Urea</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FEFundsRate</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Bono 2</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Bono 10</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>ICC Michigan</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Dow Jones</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -472,10 +497,25 @@
         <v>1.6093726</v>
       </c>
       <c r="N2">
-        <v>423.75</v>
+        <v>250.625</v>
       </c>
       <c r="O2">
-        <v>250.625</v>
+        <v>0.12</v>
+      </c>
+      <c r="P2">
+        <v>0.64</v>
+      </c>
+      <c r="Q2">
+        <v>2.07</v>
+      </c>
+      <c r="R2">
+        <v>90</v>
+      </c>
+      <c r="S2">
+        <v>4879.037</v>
+      </c>
+      <c r="T2">
+        <v>17182.28204954545</v>
       </c>
     </row>
     <row r="3">
@@ -519,10 +559,25 @@
         <v>1.61633455789</v>
       </c>
       <c r="N3">
-        <v>383.875</v>
+        <v>263.625</v>
       </c>
       <c r="O3">
-        <v>263.625</v>
+        <v>0.12</v>
+      </c>
+      <c r="P3">
+        <v>0.88</v>
+      </c>
+      <c r="Q3">
+        <v>2.26</v>
+      </c>
+      <c r="R3">
+        <v>91.3</v>
+      </c>
+      <c r="S3">
+        <v>5082.508</v>
+      </c>
+      <c r="T3">
+        <v>17724.513673</v>
       </c>
     </row>
     <row r="4">
@@ -566,10 +621,25 @@
         <v>1.7366393</v>
       </c>
       <c r="N4">
-        <v>340.625</v>
+        <v>264</v>
       </c>
       <c r="O4">
-        <v>264</v>
+        <v>0.24</v>
+      </c>
+      <c r="P4">
+        <v>0.98</v>
+      </c>
+      <c r="Q4">
+        <v>2.24</v>
+      </c>
+      <c r="R4">
+        <v>92.59999999999999</v>
+      </c>
+      <c r="S4">
+        <v>5040.54</v>
+      </c>
+      <c r="T4">
+        <v>17542.85493636364</v>
       </c>
     </row>
     <row r="5">
@@ -613,10 +683,25 @@
         <v>1.85077849</v>
       </c>
       <c r="N5">
-        <v>327.125</v>
+        <v>233.875</v>
       </c>
       <c r="O5">
-        <v>233.875</v>
+        <v>0.34</v>
+      </c>
+      <c r="P5">
+        <v>0.9</v>
+      </c>
+      <c r="Q5">
+        <v>2.09</v>
+      </c>
+      <c r="R5">
+        <v>92</v>
+      </c>
+      <c r="S5">
+        <v>4610.714</v>
+      </c>
+      <c r="T5">
+        <v>16305.25210789474</v>
       </c>
     </row>
     <row r="6">
@@ -660,10 +745,25 @@
         <v>1.76684545714</v>
       </c>
       <c r="N6">
-        <v>326</v>
+        <v>191.875</v>
       </c>
       <c r="O6">
-        <v>191.875</v>
+        <v>0.38</v>
+      </c>
+      <c r="P6">
+        <v>0.73</v>
+      </c>
+      <c r="Q6">
+        <v>1.78</v>
+      </c>
+      <c r="R6">
+        <v>91.7</v>
+      </c>
+      <c r="S6">
+        <v>4463.206</v>
+      </c>
+      <c r="T6">
+        <v>16299.8984375</v>
       </c>
     </row>
     <row r="7">
@@ -707,10 +807,25 @@
         <v>1.8548871</v>
       </c>
       <c r="N7">
-        <v>338.125</v>
+        <v>201.75</v>
       </c>
       <c r="O7">
-        <v>201.75</v>
+        <v>0.36</v>
+      </c>
+      <c r="P7">
+        <v>0.88</v>
+      </c>
+      <c r="Q7">
+        <v>1.89</v>
+      </c>
+      <c r="R7">
+        <v>91</v>
+      </c>
+      <c r="S7">
+        <v>4754.479</v>
+      </c>
+      <c r="T7">
+        <v>17302.14275636364</v>
       </c>
     </row>
     <row r="8">
@@ -754,10 +869,25 @@
         <v>1.93376668571</v>
       </c>
       <c r="N8">
-        <v>330.5</v>
+        <v>196.25</v>
       </c>
       <c r="O8">
-        <v>196.25</v>
+        <v>0.37</v>
+      </c>
+      <c r="P8">
+        <v>0.77</v>
+      </c>
+      <c r="Q8">
+        <v>1.81</v>
+      </c>
+      <c r="R8">
+        <v>89</v>
+      </c>
+      <c r="S8">
+        <v>4892.17</v>
+      </c>
+      <c r="T8">
+        <v>17844.36588619048</v>
       </c>
     </row>
     <row r="9">
@@ -801,10 +931,25 @@
         <v>2.05554569524</v>
       </c>
       <c r="N9">
-        <v>313.5</v>
+        <v>198.375</v>
       </c>
       <c r="O9">
-        <v>198.375</v>
+        <v>0.37</v>
+      </c>
+      <c r="P9">
+        <v>0.82</v>
+      </c>
+      <c r="Q9">
+        <v>1.81</v>
+      </c>
+      <c r="R9">
+        <v>94.7</v>
+      </c>
+      <c r="S9">
+        <v>4788.235</v>
+      </c>
+      <c r="T9">
+        <v>17692.32003428571</v>
       </c>
     </row>
     <row r="10">
@@ -848,10 +993,25 @@
         <v>2.154515</v>
       </c>
       <c r="N10">
-        <v>306.625</v>
+        <v>142.625</v>
       </c>
       <c r="O10">
-        <v>142.625</v>
+        <v>0.38</v>
+      </c>
+      <c r="P10">
+        <v>0.73</v>
+      </c>
+      <c r="Q10">
+        <v>1.64</v>
+      </c>
+      <c r="R10">
+        <v>93.5</v>
+      </c>
+      <c r="S10">
+        <v>4856.232</v>
+      </c>
+      <c r="T10">
+        <v>17754.86780863637</v>
       </c>
     </row>
     <row r="11">
@@ -895,10 +1055,25 @@
         <v>1.9621118</v>
       </c>
       <c r="N11">
-        <v>305.2</v>
+        <v>181</v>
       </c>
       <c r="O11">
-        <v>181</v>
+        <v>0.39</v>
+      </c>
+      <c r="P11">
+        <v>0.67</v>
+      </c>
+      <c r="Q11">
+        <v>1.5</v>
+      </c>
+      <c r="R11">
+        <v>90</v>
+      </c>
+      <c r="S11">
+        <v>5023.989</v>
+      </c>
+      <c r="T11">
+        <v>18341.182422</v>
       </c>
     </row>
     <row r="12">
@@ -942,10 +1117,25 @@
         <v>1.7416498</v>
       </c>
       <c r="N12">
-        <v>318.0625</v>
+        <v>186.25</v>
       </c>
       <c r="O12">
-        <v>186.25</v>
+        <v>0.4</v>
+      </c>
+      <c r="P12">
+        <v>0.74</v>
+      </c>
+      <c r="Q12">
+        <v>1.56</v>
+      </c>
+      <c r="R12">
+        <v>89.8</v>
+      </c>
+      <c r="S12">
+        <v>5217.038</v>
+      </c>
+      <c r="T12">
+        <v>18495.18749956522</v>
       </c>
     </row>
     <row r="13">
@@ -989,10 +1179,25 @@
         <v>1.70490613333</v>
       </c>
       <c r="N13">
-        <v>320</v>
+        <v>187.3</v>
       </c>
       <c r="O13">
-        <v>187.3</v>
+        <v>0.4</v>
+      </c>
+      <c r="P13">
+        <v>0.77</v>
+      </c>
+      <c r="Q13">
+        <v>1.63</v>
+      </c>
+      <c r="R13">
+        <v>91.2</v>
+      </c>
+      <c r="S13">
+        <v>5254.154</v>
+      </c>
+      <c r="T13">
+        <v>18267.4029952381</v>
       </c>
     </row>
     <row r="14">
@@ -1036,10 +1241,25 @@
         <v>1.5873264</v>
       </c>
       <c r="N14">
-        <v>310</v>
+        <v>187.5</v>
       </c>
       <c r="O14">
-        <v>187.5</v>
+        <v>0.4</v>
+      </c>
+      <c r="P14">
+        <v>0.84</v>
+      </c>
+      <c r="Q14">
+        <v>1.76</v>
+      </c>
+      <c r="R14">
+        <v>87.2</v>
+      </c>
+      <c r="S14">
+        <v>5255.989</v>
+      </c>
+      <c r="T14">
+        <v>18184.54641</v>
       </c>
     </row>
     <row r="15">
@@ -1083,10 +1303,25 @@
         <v>1.75597983</v>
       </c>
       <c r="N15">
-        <v>298</v>
+        <v>205</v>
       </c>
       <c r="O15">
-        <v>205</v>
+        <v>0.41</v>
+      </c>
+      <c r="P15">
+        <v>0.98</v>
+      </c>
+      <c r="Q15">
+        <v>2.14</v>
+      </c>
+      <c r="R15">
+        <v>93.8</v>
+      </c>
+      <c r="S15">
+        <v>5260.565</v>
+      </c>
+      <c r="T15">
+        <v>18697.32663761905</v>
       </c>
     </row>
     <row r="16">
@@ -1130,10 +1365,25 @@
         <v>1.86237899048</v>
       </c>
       <c r="N16">
-        <v>296.625</v>
+        <v>217.75</v>
       </c>
       <c r="O16">
-        <v>217.75</v>
+        <v>0.54</v>
+      </c>
+      <c r="P16">
+        <v>1.2</v>
+      </c>
+      <c r="Q16">
+        <v>2.49</v>
+      </c>
+      <c r="R16">
+        <v>98.2</v>
+      </c>
+      <c r="S16">
+        <v>5413.117</v>
+      </c>
+      <c r="T16">
+        <v>19712.42373619047</v>
       </c>
     </row>
     <row r="17">
@@ -1177,10 +1427,25 @@
         <v>1.9400656</v>
       </c>
       <c r="N17">
-        <v>308</v>
+        <v>233.75</v>
       </c>
       <c r="O17">
-        <v>233.75</v>
+        <v>0.65</v>
+      </c>
+      <c r="P17">
+        <v>1.21</v>
+      </c>
+      <c r="Q17">
+        <v>2.43</v>
+      </c>
+      <c r="R17">
+        <v>98.5</v>
+      </c>
+      <c r="S17">
+        <v>5561.424</v>
+      </c>
+      <c r="T17">
+        <v>19908.15254</v>
       </c>
     </row>
     <row r="18">
@@ -1224,10 +1489,25 @@
         <v>1.94116791</v>
       </c>
       <c r="N18">
-        <v>326</v>
+        <v>191.875</v>
       </c>
       <c r="O18">
-        <v>191.875</v>
+        <v>0.66</v>
+      </c>
+      <c r="P18">
+        <v>1.2</v>
+      </c>
+      <c r="Q18">
+        <v>2.42</v>
+      </c>
+      <c r="R18">
+        <v>96.3</v>
+      </c>
+      <c r="S18">
+        <v>5764.702</v>
+      </c>
+      <c r="T18">
+        <v>20424.14412</v>
       </c>
     </row>
     <row r="19">
@@ -1271,10 +1551,25 @@
         <v>2.12602050435</v>
       </c>
       <c r="N19">
-        <v>325.625</v>
+        <v>223.5</v>
       </c>
       <c r="O19">
-        <v>223.5</v>
+        <v>0.79</v>
+      </c>
+      <c r="P19">
+        <v>1.31</v>
+      </c>
+      <c r="Q19">
+        <v>2.48</v>
+      </c>
+      <c r="R19">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="S19">
+        <v>5864.964</v>
+      </c>
+      <c r="T19">
+        <v>20823.05799913044</v>
       </c>
     </row>
     <row r="20">
@@ -1318,10 +1613,25 @@
         <v>2.1605276</v>
       </c>
       <c r="N20">
-        <v>313.125</v>
+        <v>207.875</v>
       </c>
       <c r="O20">
-        <v>207.875</v>
+        <v>0.9</v>
+      </c>
+      <c r="P20">
+        <v>1.24</v>
+      </c>
+      <c r="Q20">
+        <v>2.3</v>
+      </c>
+      <c r="R20">
+        <v>97</v>
+      </c>
+      <c r="S20">
+        <v>5912.169</v>
+      </c>
+      <c r="T20">
+        <v>20684.69366842105</v>
       </c>
     </row>
     <row r="21">
@@ -1365,10 +1675,25 @@
         <v>2.334893</v>
       </c>
       <c r="N21">
-        <v>309.25</v>
+        <v>178.75</v>
       </c>
       <c r="O21">
-        <v>178.75</v>
+        <v>0.91</v>
+      </c>
+      <c r="P21">
+        <v>1.3</v>
+      </c>
+      <c r="Q21">
+        <v>2.3</v>
+      </c>
+      <c r="R21">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="S21">
+        <v>6124.878</v>
+      </c>
+      <c r="T21">
+        <v>20936.81125772727</v>
       </c>
     </row>
     <row r="22">
@@ -1412,10 +1737,25 @@
         <v>2.4341009</v>
       </c>
       <c r="N22">
-        <v>310.3</v>
+        <v>191</v>
       </c>
       <c r="O22">
-        <v>191</v>
+        <v>1.04</v>
+      </c>
+      <c r="P22">
+        <v>1.34</v>
+      </c>
+      <c r="Q22">
+        <v>2.19</v>
+      </c>
+      <c r="R22">
+        <v>95</v>
+      </c>
+      <c r="S22">
+        <v>6224.286</v>
+      </c>
+      <c r="T22">
+        <v>21317.79536636364</v>
       </c>
     </row>
     <row r="23">
@@ -1459,10 +1799,25 @@
         <v>2.34571568</v>
       </c>
       <c r="N23">
-        <v>313.75</v>
+        <v>181</v>
       </c>
       <c r="O23">
-        <v>181</v>
+        <v>1.15</v>
+      </c>
+      <c r="P23">
+        <v>1.37</v>
+      </c>
+      <c r="Q23">
+        <v>2.32</v>
+      </c>
+      <c r="R23">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="S23">
+        <v>6294.674</v>
+      </c>
+      <c r="T23">
+        <v>21581.250976</v>
       </c>
     </row>
     <row r="24">
@@ -1506,10 +1861,25 @@
         <v>2.19215910435</v>
       </c>
       <c r="N24">
-        <v>320.75</v>
+        <v>192.625</v>
       </c>
       <c r="O24">
-        <v>192.625</v>
+        <v>1.16</v>
+      </c>
+      <c r="P24">
+        <v>1.34</v>
+      </c>
+      <c r="Q24">
+        <v>2.21</v>
+      </c>
+      <c r="R24">
+        <v>96.8</v>
+      </c>
+      <c r="S24">
+        <v>6311.397</v>
+      </c>
+      <c r="T24">
+        <v>21914.07693608696</v>
       </c>
     </row>
     <row r="25">
@@ -1553,10 +1923,25 @@
         <v>2.11423058</v>
       </c>
       <c r="N25">
-        <v>325.9</v>
+        <v>219</v>
       </c>
       <c r="O25">
-        <v>219</v>
+        <v>1.15</v>
+      </c>
+      <c r="P25">
+        <v>1.38</v>
+      </c>
+      <c r="Q25">
+        <v>2.2</v>
+      </c>
+      <c r="R25">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="S25">
+        <v>6428.079</v>
+      </c>
+      <c r="T25">
+        <v>22173.413965</v>
       </c>
     </row>
     <row r="26">
@@ -1600,10 +1985,25 @@
         <v>1.9771433</v>
       </c>
       <c r="N26">
-        <v>322.375</v>
+        <v>252.5</v>
       </c>
       <c r="O26">
-        <v>252.5</v>
+        <v>1.15</v>
+      </c>
+      <c r="P26">
+        <v>1.55</v>
+      </c>
+      <c r="Q26">
+        <v>2.36</v>
+      </c>
+      <c r="R26">
+        <v>100.7</v>
+      </c>
+      <c r="S26">
+        <v>6603.011</v>
+      </c>
+      <c r="T26">
+        <v>23036.23739409091</v>
       </c>
     </row>
     <row r="27">
@@ -1647,10 +2047,25 @@
         <v>1.9621118</v>
       </c>
       <c r="N27">
-        <v>344</v>
+        <v>280</v>
       </c>
       <c r="O27">
-        <v>280</v>
+        <v>1.16</v>
+      </c>
+      <c r="P27">
+        <v>1.7</v>
+      </c>
+      <c r="Q27">
+        <v>2.35</v>
+      </c>
+      <c r="R27">
+        <v>98.5</v>
+      </c>
+      <c r="S27">
+        <v>6796.043</v>
+      </c>
+      <c r="T27">
+        <v>23557.92940952381</v>
       </c>
     </row>
     <row r="28">
@@ -1694,10 +2109,25 @@
         <v>1.96559277895</v>
       </c>
       <c r="N28">
-        <v>357.25</v>
+        <v>214.625</v>
       </c>
       <c r="O28">
-        <v>214.625</v>
+        <v>1.3</v>
+      </c>
+      <c r="P28">
+        <v>1.84</v>
+      </c>
+      <c r="Q28">
+        <v>2.4</v>
+      </c>
+      <c r="R28">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="S28">
+        <v>6889.741</v>
+      </c>
+      <c r="T28">
+        <v>24545.3841805</v>
       </c>
     </row>
     <row r="29">
@@ -1741,10 +2171,25 @@
         <v>2.07013818</v>
       </c>
       <c r="N29">
-        <v>360.375</v>
+        <v>219.625</v>
       </c>
       <c r="O29">
-        <v>219.625</v>
+        <v>1.41</v>
+      </c>
+      <c r="P29">
+        <v>2.03</v>
+      </c>
+      <c r="Q29">
+        <v>2.58</v>
+      </c>
+      <c r="R29">
+        <v>95.7</v>
+      </c>
+      <c r="S29">
+        <v>7279.498</v>
+      </c>
+      <c r="T29">
+        <v>25804.0177652381</v>
       </c>
     </row>
     <row r="30">
@@ -1788,10 +2233,25 @@
         <v>1.984158</v>
       </c>
       <c r="N30">
-        <v>370</v>
+        <v>232.5</v>
       </c>
       <c r="O30">
-        <v>232.5</v>
+        <v>1.42</v>
+      </c>
+      <c r="P30">
+        <v>2.18</v>
+      </c>
+      <c r="Q30">
+        <v>2.86</v>
+      </c>
+      <c r="R30">
+        <v>99.7</v>
+      </c>
+      <c r="S30">
+        <v>7161.773</v>
+      </c>
+      <c r="T30">
+        <v>24981.54523052632</v>
       </c>
     </row>
     <row r="31">
@@ -1835,10 +2295,25 @@
         <v>2.2010374925</v>
       </c>
       <c r="N31">
-        <v>378</v>
+        <v>232.5</v>
       </c>
       <c r="O31">
-        <v>232.5</v>
+        <v>1.51</v>
+      </c>
+      <c r="P31">
+        <v>2.28</v>
+      </c>
+      <c r="Q31">
+        <v>2.84</v>
+      </c>
+      <c r="R31">
+        <v>101.4</v>
+      </c>
+      <c r="S31">
+        <v>7311.506</v>
+      </c>
+      <c r="T31">
+        <v>24582.17038904762</v>
       </c>
     </row>
     <row r="32">
@@ -1882,10 +2357,25 @@
         <v>2.362470792</v>
       </c>
       <c r="N32">
-        <v>384.75</v>
+        <v>230.625</v>
       </c>
       <c r="O32">
-        <v>230.625</v>
+        <v>1.69</v>
+      </c>
+      <c r="P32">
+        <v>2.38</v>
+      </c>
+      <c r="Q32">
+        <v>2.87</v>
+      </c>
+      <c r="R32">
+        <v>98.8</v>
+      </c>
+      <c r="S32">
+        <v>7084.142</v>
+      </c>
+      <c r="T32">
+        <v>24304.21289047619</v>
       </c>
     </row>
     <row r="33">
@@ -1929,10 +2419,25 @@
         <v>2.64995324</v>
       </c>
       <c r="N33">
-        <v>384.375</v>
+        <v>221.875</v>
       </c>
       <c r="O33">
-        <v>221.875</v>
+        <v>1.7</v>
+      </c>
+      <c r="P33">
+        <v>2.51</v>
+      </c>
+      <c r="Q33">
+        <v>2.98</v>
+      </c>
+      <c r="R33">
+        <v>98</v>
+      </c>
+      <c r="S33">
+        <v>7339.327</v>
+      </c>
+      <c r="T33">
+        <v>24572.53222727273</v>
       </c>
     </row>
     <row r="34">
@@ -1976,10 +2481,25 @@
         <v>2.7227057</v>
       </c>
       <c r="N34">
-        <v>391.6</v>
+        <v>224</v>
       </c>
       <c r="O34">
-        <v>224</v>
+        <v>1.82</v>
+      </c>
+      <c r="P34">
+        <v>2.53</v>
+      </c>
+      <c r="Q34">
+        <v>2.91</v>
+      </c>
+      <c r="R34">
+        <v>98.2</v>
+      </c>
+      <c r="S34">
+        <v>7645.139</v>
+      </c>
+      <c r="T34">
+        <v>24790.10835333333</v>
       </c>
     </row>
     <row r="35">
@@ -2023,10 +2543,25 @@
         <v>2.53200607</v>
       </c>
       <c r="N35">
-        <v>400.75</v>
+        <v>252.5</v>
       </c>
       <c r="O35">
-        <v>252.5</v>
+        <v>1.91</v>
+      </c>
+      <c r="P35">
+        <v>2.61</v>
+      </c>
+      <c r="Q35">
+        <v>2.89</v>
+      </c>
+      <c r="R35">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="S35">
+        <v>7756.864</v>
+      </c>
+      <c r="T35">
+        <v>24978.23130619048</v>
       </c>
     </row>
     <row r="36">
@@ -2070,10 +2605,25 @@
         <v>2.22115465</v>
       </c>
       <c r="N36">
-        <v>409</v>
+        <v>260</v>
       </c>
       <c r="O36">
-        <v>260</v>
+        <v>1.91</v>
+      </c>
+      <c r="P36">
+        <v>2.64</v>
+      </c>
+      <c r="Q36">
+        <v>2.89</v>
+      </c>
+      <c r="R36">
+        <v>96.2</v>
+      </c>
+      <c r="S36">
+        <v>7892.233</v>
+      </c>
+      <c r="T36">
+        <v>25629.98828173913</v>
       </c>
     </row>
     <row r="37">
@@ -2117,10 +2667,25 @@
         <v>2.0282504</v>
       </c>
       <c r="N37">
-        <v>421.63</v>
+        <v>267.5</v>
       </c>
       <c r="O37">
-        <v>267.5</v>
+        <v>1.95</v>
+      </c>
+      <c r="P37">
+        <v>2.77</v>
+      </c>
+      <c r="Q37">
+        <v>3</v>
+      </c>
+      <c r="R37">
+        <v>100.1</v>
+      </c>
+      <c r="S37">
+        <v>7983.307</v>
+      </c>
+      <c r="T37">
+        <v>26232.66796894737</v>
       </c>
     </row>
     <row r="38">
@@ -2164,10 +2729,25 @@
         <v>2.0282504</v>
       </c>
       <c r="N38">
-        <v>420.75</v>
+        <v>270</v>
       </c>
       <c r="O38">
-        <v>270</v>
+        <v>2.19</v>
+      </c>
+      <c r="P38">
+        <v>2.86</v>
+      </c>
+      <c r="Q38">
+        <v>3.15</v>
+      </c>
+      <c r="R38">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="S38">
+        <v>7527.084</v>
+      </c>
+      <c r="T38">
+        <v>25609.34188217391</v>
       </c>
     </row>
     <row r="39">
@@ -2211,10 +2791,25 @@
         <v>2.0282504</v>
       </c>
       <c r="N39">
-        <v>410.2</v>
+        <v>305.6</v>
       </c>
       <c r="O39">
-        <v>305.6</v>
+        <v>2.2</v>
+      </c>
+      <c r="P39">
+        <v>2.86</v>
+      </c>
+      <c r="Q39">
+        <v>3.12</v>
+      </c>
+      <c r="R39">
+        <v>97.5</v>
+      </c>
+      <c r="S39">
+        <v>7236.081</v>
+      </c>
+      <c r="T39">
+        <v>25258.67531571428</v>
       </c>
     </row>
     <row r="40">
@@ -2258,10 +2853,25 @@
         <v>2.0879074172</v>
       </c>
       <c r="N40">
-        <v>389.67</v>
+        <v>276.67</v>
       </c>
       <c r="O40">
-        <v>276.67</v>
+        <v>2.27</v>
+      </c>
+      <c r="P40">
+        <v>2.68</v>
+      </c>
+      <c r="Q40">
+        <v>2.83</v>
+      </c>
+      <c r="R40">
+        <v>98.3</v>
+      </c>
+      <c r="S40">
+        <v>6814.292</v>
+      </c>
+      <c r="T40">
+        <v>23805.54523105263</v>
       </c>
     </row>
     <row r="41">
@@ -2305,10 +2915,25 @@
         <v>2.1495045</v>
       </c>
       <c r="N41">
-        <v>382.13</v>
+        <v>260</v>
       </c>
       <c r="O41">
-        <v>260</v>
+        <v>2.4</v>
+      </c>
+      <c r="P41">
+        <v>2.54</v>
+      </c>
+      <c r="Q41">
+        <v>2.71</v>
+      </c>
+      <c r="R41">
+        <v>91.2</v>
+      </c>
+      <c r="S41">
+        <v>6979.656</v>
+      </c>
+      <c r="T41">
+        <v>24157.79510761905</v>
       </c>
     </row>
     <row r="42">
@@ -2352,10 +2977,25 @@
         <v>2.08557052</v>
       </c>
       <c r="N42">
-        <v>357.38</v>
+        <v>250.63</v>
       </c>
       <c r="O42">
-        <v>250.63</v>
+        <v>2.4</v>
+      </c>
+      <c r="P42">
+        <v>2.5</v>
+      </c>
+      <c r="Q42">
+        <v>2.68</v>
+      </c>
+      <c r="R42">
+        <v>93.8</v>
+      </c>
+      <c r="S42">
+        <v>7430.077</v>
+      </c>
+      <c r="T42">
+        <v>25605.52683105263</v>
       </c>
     </row>
     <row r="43">
@@ -2399,10 +3039,25 @@
         <v>2.06903587</v>
       </c>
       <c r="N43">
-        <v>335.03</v>
+        <v>247.5</v>
       </c>
       <c r="O43">
-        <v>247.5</v>
+        <v>2.41</v>
+      </c>
+      <c r="P43">
+        <v>2.41</v>
+      </c>
+      <c r="Q43">
+        <v>2.57</v>
+      </c>
+      <c r="R43">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="S43">
+        <v>7629.367</v>
+      </c>
+      <c r="T43">
+        <v>25722.62118714286</v>
       </c>
     </row>
     <row r="44">
@@ -2446,10 +3101,25 @@
         <v>2.094389</v>
       </c>
       <c r="N44">
-        <v>323.75</v>
+        <v>247.5</v>
       </c>
       <c r="O44">
-        <v>247.5</v>
+        <v>2.42</v>
+      </c>
+      <c r="P44">
+        <v>2.34</v>
+      </c>
+      <c r="Q44">
+        <v>2.53</v>
+      </c>
+      <c r="R44">
+        <v>97.2</v>
+      </c>
+      <c r="S44">
+        <v>7993.369</v>
+      </c>
+      <c r="T44">
+        <v>26401.57738142857</v>
       </c>
     </row>
     <row r="45">
@@ -2493,10 +3163,25 @@
         <v>2.08667283</v>
       </c>
       <c r="N45">
-        <v>313.4</v>
+        <v>247.5</v>
       </c>
       <c r="O45">
-        <v>247.5</v>
+        <v>2.39</v>
+      </c>
+      <c r="P45">
+        <v>2.21</v>
+      </c>
+      <c r="Q45">
+        <v>2.4</v>
+      </c>
+      <c r="R45">
+        <v>100</v>
+      </c>
+      <c r="S45">
+        <v>7804.821</v>
+      </c>
+      <c r="T45">
+        <v>25744.78853</v>
       </c>
     </row>
     <row r="46">
@@ -2540,10 +3225,25 @@
         <v>2.0723428</v>
       </c>
       <c r="N46">
-        <v>314.88</v>
+        <v>247.5</v>
       </c>
       <c r="O46">
-        <v>247.5</v>
+        <v>2.38</v>
+      </c>
+      <c r="P46">
+        <v>1.81</v>
+      </c>
+      <c r="Q46">
+        <v>2.07</v>
+      </c>
+      <c r="R46">
+        <v>98.2</v>
+      </c>
+      <c r="S46">
+        <v>7825.459</v>
+      </c>
+      <c r="T46">
+        <v>26160.1008795</v>
       </c>
     </row>
     <row r="47">
@@ -2587,10 +3287,25 @@
         <v>1.98856724</v>
       </c>
       <c r="N47">
-        <v>307.5</v>
+        <v>263.5</v>
       </c>
       <c r="O47">
-        <v>263.5</v>
+        <v>2.4</v>
+      </c>
+      <c r="P47">
+        <v>1.84</v>
+      </c>
+      <c r="Q47">
+        <v>2.06</v>
+      </c>
+      <c r="R47">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="S47">
+        <v>8205.599</v>
+      </c>
+      <c r="T47">
+        <v>27089.18670136364</v>
       </c>
     </row>
     <row r="48">
@@ -2634,10 +3349,25 @@
         <v>1.90038244</v>
       </c>
       <c r="N48">
-        <v>292.9</v>
+        <v>262.5</v>
       </c>
       <c r="O48">
-        <v>262.5</v>
+        <v>2.13</v>
+      </c>
+      <c r="P48">
+        <v>1.57</v>
+      </c>
+      <c r="Q48">
+        <v>1.63</v>
+      </c>
+      <c r="R48">
+        <v>89.8</v>
+      </c>
+      <c r="S48">
+        <v>7910.933</v>
+      </c>
+      <c r="T48">
+        <v>26057.72807136364</v>
       </c>
     </row>
     <row r="49">
@@ -2681,10 +3411,25 @@
         <v>1.85298311</v>
       </c>
       <c r="N49">
-        <v>285.75</v>
+        <v>237.75</v>
       </c>
       <c r="O49">
-        <v>237.75</v>
+        <v>2.04</v>
+      </c>
+      <c r="P49">
+        <v>1.65</v>
+      </c>
+      <c r="Q49">
+        <v>1.7</v>
+      </c>
+      <c r="R49">
+        <v>93.2</v>
+      </c>
+      <c r="S49">
+        <v>8087.7</v>
+      </c>
+      <c r="T49">
+        <v>26900.2139645</v>
       </c>
     </row>
     <row r="50">
@@ -2728,10 +3473,25 @@
         <v>1.8518808</v>
       </c>
       <c r="N50">
-        <v>277.38</v>
+        <v>237</v>
       </c>
       <c r="O50">
-        <v>237</v>
+        <v>1.83</v>
+      </c>
+      <c r="P50">
+        <v>1.55</v>
+      </c>
+      <c r="Q50">
+        <v>1.71</v>
+      </c>
+      <c r="R50">
+        <v>95.5</v>
+      </c>
+      <c r="S50">
+        <v>8079.274</v>
+      </c>
+      <c r="T50">
+        <v>26736.79772434783</v>
       </c>
     </row>
     <row r="51">
@@ -2775,10 +3535,25 @@
         <v>1.8518808</v>
       </c>
       <c r="N51">
-        <v>248</v>
+        <v>224.5</v>
       </c>
       <c r="O51">
-        <v>224.5</v>
+        <v>1.55</v>
+      </c>
+      <c r="P51">
+        <v>1.61</v>
+      </c>
+      <c r="Q51">
+        <v>1.81</v>
+      </c>
+      <c r="R51">
+        <v>96.8</v>
+      </c>
+      <c r="S51">
+        <v>8517.578</v>
+      </c>
+      <c r="T51">
+        <v>27797.0460935</v>
       </c>
     </row>
     <row r="52">
@@ -2822,10 +3597,25 @@
         <v>1.97754414</v>
       </c>
       <c r="N52">
-        <v>238.16</v>
+        <v>217.5</v>
       </c>
       <c r="O52">
-        <v>217.5</v>
+        <v>1.55</v>
+      </c>
+      <c r="P52">
+        <v>1.61</v>
+      </c>
+      <c r="Q52">
+        <v>1.86</v>
+      </c>
+      <c r="R52">
+        <v>99.3</v>
+      </c>
+      <c r="S52">
+        <v>8778.591</v>
+      </c>
+      <c r="T52">
+        <v>28167.00576761905</v>
       </c>
     </row>
     <row r="53">
@@ -2869,10 +3659,25 @@
         <v>2.07124049</v>
       </c>
       <c r="N53">
-        <v>264.9</v>
+        <v>215.4</v>
       </c>
       <c r="O53">
-        <v>215.4</v>
+        <v>1.55</v>
+      </c>
+      <c r="P53">
+        <v>1.52</v>
+      </c>
+      <c r="Q53">
+        <v>1.76</v>
+      </c>
+      <c r="R53">
+        <v>99.8</v>
+      </c>
+      <c r="S53">
+        <v>9233.360000000001</v>
+      </c>
+      <c r="T53">
+        <v>28879.99432619048</v>
       </c>
     </row>
     <row r="54">
@@ -2916,10 +3721,25 @@
         <v>1.87613162</v>
       </c>
       <c r="N54">
-        <v>279.38</v>
+        <v>214.38</v>
       </c>
       <c r="O54">
-        <v>214.38</v>
+        <v>1.58</v>
+      </c>
+      <c r="P54">
+        <v>1.33</v>
+      </c>
+      <c r="Q54">
+        <v>1.5</v>
+      </c>
+      <c r="R54">
+        <v>101</v>
+      </c>
+      <c r="S54">
+        <v>9418.849</v>
+      </c>
+      <c r="T54">
+        <v>28519.73160052632</v>
       </c>
     </row>
     <row r="55">
@@ -2963,10 +3783,25 @@
         <v>1.77692372</v>
       </c>
       <c r="N55">
-        <v>276.22</v>
+        <v>231.13</v>
       </c>
       <c r="O55">
-        <v>231.13</v>
+        <v>0.65</v>
+      </c>
+      <c r="P55">
+        <v>0.45</v>
+      </c>
+      <c r="Q55">
+        <v>0.87</v>
+      </c>
+      <c r="R55">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="S55">
+        <v>7772.206</v>
+      </c>
+      <c r="T55">
+        <v>22637.42081045455</v>
       </c>
     </row>
     <row r="56">
@@ -3010,10 +3845,25 @@
         <v>1.2676565</v>
       </c>
       <c r="N56">
-        <v>282</v>
+        <v>235</v>
       </c>
       <c r="O56">
-        <v>235</v>
+        <v>0.05</v>
+      </c>
+      <c r="P56">
+        <v>0.22</v>
+      </c>
+      <c r="Q56">
+        <v>0.66</v>
+      </c>
+      <c r="R56">
+        <v>71.8</v>
+      </c>
+      <c r="S56">
+        <v>8292.406999999999</v>
+      </c>
+      <c r="T56">
+        <v>23293.89983285714</v>
       </c>
     </row>
     <row r="57">
@@ -3057,10 +3907,25 @@
         <v>1.51788087</v>
       </c>
       <c r="N57">
-        <v>263</v>
+        <v>201.9</v>
       </c>
       <c r="O57">
-        <v>201.9</v>
+        <v>0.05</v>
+      </c>
+      <c r="P57">
+        <v>0.17</v>
+      </c>
+      <c r="Q57">
+        <v>0.67</v>
+      </c>
+      <c r="R57">
+        <v>72.3</v>
+      </c>
+      <c r="S57">
+        <v>9105.656000000001</v>
+      </c>
+      <c r="T57">
+        <v>24271.0213875</v>
       </c>
     </row>
     <row r="58">
@@ -3104,10 +3969,25 @@
         <v>1.5652802</v>
       </c>
       <c r="N58">
-        <v>273</v>
+        <v>202</v>
       </c>
       <c r="O58">
-        <v>202</v>
+        <v>0.08</v>
+      </c>
+      <c r="P58">
+        <v>0.19</v>
+      </c>
+      <c r="Q58">
+        <v>0.73</v>
+      </c>
+      <c r="R58">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="S58">
+        <v>9839.969999999999</v>
+      </c>
+      <c r="T58">
+        <v>26062.27015272727</v>
       </c>
     </row>
     <row r="59">
@@ -3151,10 +4031,25 @@
         <v>1.52339242</v>
       </c>
       <c r="N59">
-        <v>305.1</v>
+        <v>214.4</v>
       </c>
       <c r="O59">
-        <v>214.4</v>
+        <v>0.09</v>
+      </c>
+      <c r="P59">
+        <v>0.15</v>
+      </c>
+      <c r="Q59">
+        <v>0.62</v>
+      </c>
+      <c r="R59">
+        <v>72.5</v>
+      </c>
+      <c r="S59">
+        <v>10499.863</v>
+      </c>
+      <c r="T59">
+        <v>26385.83087727273</v>
       </c>
     </row>
     <row r="60">
@@ -3198,10 +4093,25 @@
         <v>1.496496056</v>
       </c>
       <c r="N60">
-        <v>341.88</v>
+        <v>249.5</v>
       </c>
       <c r="O60">
-        <v>249.5</v>
+        <v>0.1</v>
+      </c>
+      <c r="P60">
+        <v>0.14</v>
+      </c>
+      <c r="Q60">
+        <v>0.65</v>
+      </c>
+      <c r="R60">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="S60">
+        <v>11212.29</v>
+      </c>
+      <c r="T60">
+        <v>27821.36728</v>
       </c>
     </row>
     <row r="61">
@@ -3242,10 +4152,25 @@
         <v>1.47158385</v>
       </c>
       <c r="N61">
-        <v>358.38</v>
+        <v>250.5</v>
       </c>
       <c r="O61">
-        <v>250.5</v>
+        <v>0.09</v>
+      </c>
+      <c r="P61">
+        <v>0.13</v>
+      </c>
+      <c r="Q61">
+        <v>0.68</v>
+      </c>
+      <c r="R61">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="S61">
+        <v>11088.74</v>
+      </c>
+      <c r="T61">
+        <v>27733.39639285714</v>
       </c>
     </row>
     <row r="62">
@@ -3286,10 +4211,25 @@
         <v>1.50134622</v>
       </c>
       <c r="N62">
-        <v>357.1</v>
+        <v>245</v>
       </c>
       <c r="O62">
-        <v>245</v>
+        <v>0.09</v>
+      </c>
+      <c r="P62">
+        <v>0.15</v>
+      </c>
+      <c r="Q62">
+        <v>0.79</v>
+      </c>
+      <c r="R62">
+        <v>81.8</v>
+      </c>
+      <c r="S62">
+        <v>11435.293</v>
+      </c>
+      <c r="T62">
+        <v>28005.10502590909</v>
       </c>
     </row>
     <row r="63">
@@ -3330,10 +4270,25 @@
         <v>1.704612184</v>
       </c>
       <c r="N63">
-        <v>359.63</v>
+        <v>245</v>
       </c>
       <c r="O63">
-        <v>245</v>
+        <v>0.09</v>
+      </c>
+      <c r="P63">
+        <v>0.17</v>
+      </c>
+      <c r="Q63">
+        <v>0.87</v>
+      </c>
+      <c r="R63">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="S63">
+        <v>11794.516</v>
+      </c>
+      <c r="T63">
+        <v>29124.036621</v>
       </c>
     </row>
     <row r="64">
@@ -3374,10 +4329,25 @@
         <v>1.8077884</v>
       </c>
       <c r="N64">
-        <v>388.5</v>
+        <v>245</v>
       </c>
       <c r="O64">
-        <v>245</v>
+        <v>0.09</v>
+      </c>
+      <c r="P64">
+        <v>0.14</v>
+      </c>
+      <c r="Q64">
+        <v>0.93</v>
+      </c>
+      <c r="R64">
+        <v>80.7</v>
+      </c>
+      <c r="S64">
+        <v>12619.051</v>
+      </c>
+      <c r="T64">
+        <v>30148.57990090909</v>
       </c>
     </row>
     <row r="65">
@@ -3418,10 +4388,25 @@
         <v>1.8077884</v>
       </c>
       <c r="N65">
-        <v>421.3</v>
+        <v>265</v>
       </c>
       <c r="O65">
-        <v>265</v>
+        <v>0.09</v>
+      </c>
+      <c r="P65">
+        <v>0.13</v>
+      </c>
+      <c r="Q65">
+        <v>1.08</v>
+      </c>
+      <c r="R65">
+        <v>79</v>
+      </c>
+      <c r="S65">
+        <v>13186.606</v>
+      </c>
+      <c r="T65">
+        <v>30821.35259052632</v>
       </c>
     </row>
     <row r="66">
@@ -3462,10 +4447,25 @@
         <v>1.8077884</v>
       </c>
       <c r="N66">
-        <v>528.88</v>
+        <v>335</v>
       </c>
       <c r="O66">
-        <v>335</v>
+        <v>0.08</v>
+      </c>
+      <c r="P66">
+        <v>0.12</v>
+      </c>
+      <c r="Q66">
+        <v>1.26</v>
+      </c>
+      <c r="R66">
+        <v>76.8</v>
+      </c>
+      <c r="S66">
+        <v>13737.405</v>
+      </c>
+      <c r="T66">
+        <v>31283.90984842105</v>
       </c>
     </row>
     <row r="67">
@@ -3506,10 +4506,25 @@
         <v>1.886272872</v>
       </c>
       <c r="N67">
-        <v>534.13</v>
+        <v>352.88</v>
       </c>
       <c r="O67">
-        <v>352.88</v>
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P67">
+        <v>0.15</v>
+      </c>
+      <c r="Q67">
+        <v>1.61</v>
+      </c>
+      <c r="R67">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="S67">
+        <v>13168.811</v>
+      </c>
+      <c r="T67">
+        <v>32373.29110043478</v>
       </c>
     </row>
     <row r="68">
@@ -3550,10 +4565,25 @@
         <v>2.26414474</v>
       </c>
       <c r="N68">
-        <v>543.4</v>
+        <v>328.1</v>
       </c>
       <c r="O68">
-        <v>328.1</v>
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P68">
+        <v>0.16</v>
+      </c>
+      <c r="Q68">
+        <v>1.64</v>
+      </c>
+      <c r="R68">
+        <v>88.3</v>
+      </c>
+      <c r="S68">
+        <v>13900.438</v>
+      </c>
+      <c r="T68">
+        <v>33803.28608714286</v>
       </c>
     </row>
     <row r="69">
@@ -3594,10 +4624,25 @@
         <v>2.374816664</v>
       </c>
       <c r="N69">
-        <v>574.63</v>
+        <v>331.63</v>
       </c>
       <c r="O69">
-        <v>331.63</v>
+        <v>0.06</v>
+      </c>
+      <c r="P69">
+        <v>0.16</v>
+      </c>
+      <c r="Q69">
+        <v>1.62</v>
+      </c>
+      <c r="R69">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="S69">
+        <v>13520.229</v>
+      </c>
+      <c r="T69">
+        <v>34270.3085945</v>
       </c>
     </row>
     <row r="70">
@@ -3638,10 +4683,25 @@
         <v>2.3809896</v>
       </c>
       <c r="N70">
-        <v>604.75</v>
+        <v>393.25</v>
       </c>
       <c r="O70">
-        <v>393.25</v>
+        <v>0.08</v>
+      </c>
+      <c r="P70">
+        <v>0.2</v>
+      </c>
+      <c r="Q70">
+        <v>1.52</v>
+      </c>
+      <c r="R70">
+        <v>85.5</v>
+      </c>
+      <c r="S70">
+        <v>14097.169</v>
+      </c>
+      <c r="T70">
+        <v>34289.90678318182</v>
       </c>
     </row>
     <row r="71">
@@ -3682,10 +4742,25 @@
         <v>2.3809896</v>
       </c>
       <c r="N71">
-        <v>613</v>
+        <v>441.5</v>
       </c>
       <c r="O71">
-        <v>441.5</v>
+        <v>0.1</v>
+      </c>
+      <c r="P71">
+        <v>0.22</v>
+      </c>
+      <c r="Q71">
+        <v>1.32</v>
+      </c>
+      <c r="R71">
+        <v>81.2</v>
+      </c>
+      <c r="S71">
+        <v>14639.073</v>
+      </c>
+      <c r="T71">
+        <v>34798.8043147619</v>
       </c>
     </row>
     <row r="72">
@@ -3726,10 +4801,25 @@
         <v>2.3809896</v>
       </c>
       <c r="N72">
-        <v>603.13</v>
+        <v>446.88</v>
       </c>
       <c r="O72">
-        <v>446.88</v>
+        <v>0.09</v>
+      </c>
+      <c r="P72">
+        <v>0.22</v>
+      </c>
+      <c r="Q72">
+        <v>1.28</v>
+      </c>
+      <c r="R72">
+        <v>70.3</v>
+      </c>
+      <c r="S72">
+        <v>14856.518</v>
+      </c>
+      <c r="T72">
+        <v>35243.96591</v>
       </c>
     </row>
     <row r="73">
@@ -3770,10 +4860,25 @@
         <v>1.832465</v>
       </c>
       <c r="N73">
-        <v>643.75</v>
+        <v>418.75</v>
       </c>
       <c r="O73">
-        <v>418.75</v>
+        <v>0.08</v>
+      </c>
+      <c r="P73">
+        <v>0.24</v>
+      </c>
+      <c r="Q73">
+        <v>1.37</v>
+      </c>
+      <c r="R73">
+        <v>72.8</v>
+      </c>
+      <c r="S73">
+        <v>15023.539</v>
+      </c>
+      <c r="T73">
+        <v>34688.42131666667</v>
       </c>
     </row>
     <row r="74">
@@ -3811,10 +4916,25 @@
         <v>1.75807</v>
       </c>
       <c r="N74">
-        <v>672.9</v>
+        <v>695</v>
       </c>
       <c r="O74">
-        <v>695</v>
+        <v>0.08</v>
+      </c>
+      <c r="P74">
+        <v>0.39</v>
+      </c>
+      <c r="Q74">
+        <v>1.58</v>
+      </c>
+      <c r="R74">
+        <v>71.7</v>
+      </c>
+      <c r="S74">
+        <v>14879.012</v>
+      </c>
+      <c r="T74">
+        <v>35055.51785761904</v>
       </c>
     </row>
     <row r="75">
@@ -3855,10 +4975,25 @@
         <v>1.551674</v>
       </c>
       <c r="N75">
-        <v>726.6900000000001</v>
+        <v>900.5</v>
       </c>
       <c r="O75">
-        <v>900.5</v>
+        <v>0.08</v>
+      </c>
+      <c r="P75">
+        <v>0.51</v>
+      </c>
+      <c r="Q75">
+        <v>1.56</v>
+      </c>
+      <c r="R75">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="S75">
+        <v>15814.933</v>
+      </c>
+      <c r="T75">
+        <v>35848.5706852381</v>
       </c>
     </row>
     <row r="76">
@@ -3899,10 +5034,25 @@
         <v>1.471808</v>
       </c>
       <c r="N76">
-        <v>745</v>
+        <v>890</v>
       </c>
       <c r="O76">
-        <v>890</v>
+        <v>0.08</v>
+      </c>
+      <c r="P76">
+        <v>0.68</v>
+      </c>
+      <c r="Q76">
+        <v>1.47</v>
+      </c>
+      <c r="R76">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="S76">
+        <v>15474.432</v>
+      </c>
+      <c r="T76">
+        <v>35641.33380863637</v>
       </c>
     </row>
     <row r="77">
@@ -3943,10 +5093,25 @@
         <v>1.3575</v>
       </c>
       <c r="N77">
-        <v>699.38</v>
+        <v>846.38</v>
       </c>
       <c r="O77">
-        <v>846.38</v>
+        <v>0.08</v>
+      </c>
+      <c r="P77">
+        <v>0.98</v>
+      </c>
+      <c r="Q77">
+        <v>1.76</v>
+      </c>
+      <c r="R77">
+        <v>67.2</v>
+      </c>
+      <c r="S77">
+        <v>14531.378</v>
+      </c>
+      <c r="T77">
+        <v>35456.1447265</v>
       </c>
     </row>
     <row r="78">
@@ -3987,10 +5152,25 @@
         <v>1.448352</v>
       </c>
       <c r="N78">
-        <v>747.13</v>
+        <v>744.17</v>
       </c>
       <c r="O78">
-        <v>744.17</v>
+        <v>0.08</v>
+      </c>
+      <c r="P78">
+        <v>1.44</v>
+      </c>
+      <c r="Q78">
+        <v>1.93</v>
+      </c>
+      <c r="R78">
+        <v>62.8</v>
+      </c>
+      <c r="S78">
+        <v>13898.728</v>
+      </c>
+      <c r="T78">
+        <v>34648.48026368421</v>
       </c>
     </row>
     <row r="79">
@@ -4031,10 +5211,25 @@
         <v>1.756807</v>
       </c>
       <c r="N79">
-        <v>938.13</v>
+        <v>872.5</v>
       </c>
       <c r="O79">
-        <v>872.5</v>
+        <v>0.2</v>
+      </c>
+      <c r="P79">
+        <v>1.91</v>
+      </c>
+      <c r="Q79">
+        <v>2.13</v>
+      </c>
+      <c r="R79">
+        <v>59.4</v>
+      </c>
+      <c r="S79">
+        <v>13623.263</v>
+      </c>
+      <c r="T79">
+        <v>34029.74065956522</v>
       </c>
     </row>
     <row r="80">
@@ -4075,10 +5270,25 @@
         <v>1.868574</v>
       </c>
       <c r="N80">
-        <v>954</v>
+        <v>925</v>
       </c>
       <c r="O80">
-        <v>925</v>
+        <v>0.33</v>
+      </c>
+      <c r="P80">
+        <v>2.54</v>
+      </c>
+      <c r="Q80">
+        <v>2.75</v>
+      </c>
+      <c r="R80">
+        <v>65.2</v>
+      </c>
+      <c r="S80">
+        <v>13394.163</v>
+      </c>
+      <c r="T80">
+        <v>34314.9900405</v>
       </c>
     </row>
     <row r="81">
@@ -4119,10 +5329,25 @@
         <v>1.895698</v>
       </c>
       <c r="N81">
-        <v>842.5</v>
+        <v>707.5</v>
       </c>
       <c r="O81">
-        <v>707.5</v>
+        <v>0.77</v>
+      </c>
+      <c r="P81">
+        <v>2.62</v>
+      </c>
+      <c r="Q81">
+        <v>2.9</v>
+      </c>
+      <c r="R81">
+        <v>58.4</v>
+      </c>
+      <c r="S81">
+        <v>11829.73</v>
+      </c>
+      <c r="T81">
+        <v>32379.46279666667</v>
       </c>
     </row>
     <row r="82">
@@ -4163,10 +5388,25 @@
         <v>1.848386</v>
       </c>
       <c r="N82">
-        <v>783.75</v>
+        <v>690</v>
       </c>
       <c r="O82">
-        <v>690</v>
+        <v>1.21</v>
+      </c>
+      <c r="P82">
+        <v>3</v>
+      </c>
+      <c r="Q82">
+        <v>3.14</v>
+      </c>
+      <c r="R82">
+        <v>50</v>
+      </c>
+      <c r="S82">
+        <v>11418.919</v>
+      </c>
+      <c r="T82">
+        <v>31446.71279857143</v>
       </c>
     </row>
     <row r="83">
@@ -4207,10 +5447,25 @@
         <v>1.723275</v>
       </c>
       <c r="N83">
-        <v>784</v>
+        <v>601</v>
       </c>
       <c r="O83">
-        <v>601</v>
+        <v>1.68</v>
+      </c>
+      <c r="P83">
+        <v>3.04</v>
+      </c>
+      <c r="Q83">
+        <v>2.9</v>
+      </c>
+      <c r="R83">
+        <v>51.5</v>
+      </c>
+      <c r="S83">
+        <v>11622.632</v>
+      </c>
+      <c r="T83">
+        <v>31535.3233395</v>
       </c>
     </row>
     <row r="84">
@@ -4248,10 +5503,25 @@
         <v>1.835136</v>
       </c>
       <c r="N84">
-        <v>749.38</v>
+        <v>591.25</v>
       </c>
       <c r="O84">
-        <v>591.25</v>
+        <v>2.33</v>
+      </c>
+      <c r="P84">
+        <v>3.25</v>
+      </c>
+      <c r="Q84">
+        <v>2.9</v>
+      </c>
+      <c r="R84">
+        <v>58.2</v>
+      </c>
+      <c r="S84">
+        <v>12570.26</v>
+      </c>
+      <c r="T84">
+        <v>33009.56487782609</v>
       </c>
     </row>
     <row r="85">
@@ -4289,10 +5559,25 @@
         <v>1.74956</v>
       </c>
       <c r="N85">
-        <v>752</v>
+        <v>678</v>
       </c>
       <c r="O85">
-        <v>678</v>
+        <v>2.56</v>
+      </c>
+      <c r="P85">
+        <v>3.86</v>
+      </c>
+      <c r="Q85">
+        <v>3.52</v>
+      </c>
+      <c r="R85">
+        <v>58.6</v>
+      </c>
+      <c r="S85">
+        <v>11402.85</v>
+      </c>
+      <c r="T85">
+        <v>30649.55952380952</v>
       </c>
     </row>
     <row r="86">
@@ -4330,10 +5615,25 @@
         <v>1.62792</v>
       </c>
       <c r="N86">
-        <v>725</v>
+        <v>636.25</v>
       </c>
       <c r="O86">
-        <v>636.25</v>
+        <v>3.08</v>
+      </c>
+      <c r="P86">
+        <v>4.38</v>
+      </c>
+      <c r="Q86">
+        <v>3.98</v>
+      </c>
+      <c r="R86">
+        <v>59.9</v>
+      </c>
+      <c r="S86">
+        <v>10801.494</v>
+      </c>
+      <c r="T86">
+        <v>30570.68377952381</v>
       </c>
     </row>
     <row r="87">
@@ -4371,10 +5671,25 @@
         <v>1.539822</v>
       </c>
       <c r="N87">
-        <v>665.63</v>
+        <v>588.75</v>
       </c>
       <c r="O87">
-        <v>588.75</v>
+        <v>3.78</v>
+      </c>
+      <c r="P87">
+        <v>4.5</v>
+      </c>
+      <c r="Q87">
+        <v>3.89</v>
+      </c>
+      <c r="R87">
+        <v>56.7</v>
+      </c>
+      <c r="S87">
+        <v>10973.638</v>
+      </c>
+      <c r="T87">
+        <v>33417.95824095238</v>
       </c>
     </row>
     <row r="88">
@@ -4412,10 +5727,25 @@
         <v>1.54686</v>
       </c>
       <c r="N88">
-        <v>625</v>
+        <v>519.38</v>
       </c>
       <c r="O88">
-        <v>519.38</v>
+        <v>4.1</v>
+      </c>
+      <c r="P88">
+        <v>4.29</v>
+      </c>
+      <c r="Q88">
+        <v>3.62</v>
+      </c>
+      <c r="R88">
+        <v>59.8</v>
+      </c>
+      <c r="S88">
+        <v>10838.996</v>
+      </c>
+      <c r="T88">
+        <v>33482.25725476191</v>
       </c>
     </row>
     <row r="89">
@@ -4453,10 +5783,25 @@
         <v>1.544652</v>
       </c>
       <c r="N89">
-        <v>631</v>
+        <v>443.75</v>
       </c>
       <c r="O89">
-        <v>443.75</v>
+        <v>4.33</v>
+      </c>
+      <c r="P89">
+        <v>4.21</v>
+      </c>
+      <c r="Q89">
+        <v>3.53</v>
+      </c>
+      <c r="R89">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="S89">
+        <v>11013.991</v>
+      </c>
+      <c r="T89">
+        <v>33656.0001955</v>
       </c>
     </row>
     <row r="90">
@@ -4497,10 +5842,25 @@
         <v>1.532076</v>
       </c>
       <c r="N90">
-        <v>612.5</v>
+        <v>357.5</v>
       </c>
       <c r="O90">
-        <v>357.5</v>
+        <v>4.57</v>
+      </c>
+      <c r="P90">
+        <v>4.53</v>
+      </c>
+      <c r="Q90">
+        <v>3.75</v>
+      </c>
+      <c r="R90">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="S90">
+        <v>11785.074</v>
+      </c>
+      <c r="T90">
+        <v>33648.25678526315</v>
       </c>
     </row>
     <row r="91">
@@ -4541,10 +5901,25 @@
         <v>1.522224</v>
       </c>
       <c r="N91">
-        <v>606</v>
+        <v>313.5</v>
       </c>
       <c r="O91">
-        <v>313.5</v>
+        <v>4.65</v>
+      </c>
+      <c r="P91">
+        <v>4.3</v>
+      </c>
+      <c r="Q91">
+        <v>3.66</v>
+      </c>
+      <c r="R91">
+        <v>62</v>
+      </c>
+      <c r="S91">
+        <v>11637.092</v>
+      </c>
+      <c r="T91">
+        <v>32483.47826217391</v>
       </c>
     </row>
     <row r="92">
@@ -4585,10 +5960,25 @@
         <v>1.570852</v>
       </c>
       <c r="N92">
-        <v>637</v>
+        <v>313.38</v>
       </c>
       <c r="O92">
-        <v>313.38</v>
+        <v>4.83</v>
+      </c>
+      <c r="P92">
+        <v>4.02</v>
+      </c>
+      <c r="Q92">
+        <v>3.46</v>
+      </c>
+      <c r="R92">
+        <v>63.7</v>
+      </c>
+      <c r="S92">
+        <v>12073.465</v>
+      </c>
+      <c r="T92">
+        <v>33731.2802231579</v>
       </c>
     </row>
     <row r="93">
@@ -4629,10 +6019,25 @@
         <v>1.542912</v>
       </c>
       <c r="N93">
-        <v>510</v>
+        <v>329.25</v>
       </c>
       <c r="O93">
-        <v>329.25</v>
+        <v>5.06</v>
+      </c>
+      <c r="P93">
+        <v>4.13</v>
+      </c>
+      <c r="Q93">
+        <v>3.57</v>
+      </c>
+      <c r="R93">
+        <v>59</v>
+      </c>
+      <c r="S93">
+        <v>12446.53</v>
+      </c>
+      <c r="T93">
+        <v>33316.80229136364</v>
       </c>
     </row>
     <row r="94">
@@ -4673,10 +6078,25 @@
         <v>1.467504</v>
       </c>
       <c r="N94">
-        <v>454.55</v>
+        <v>287.5</v>
       </c>
       <c r="O94">
-        <v>287.5</v>
+        <v>5.08</v>
+      </c>
+      <c r="P94">
+        <v>4.64</v>
+      </c>
+      <c r="Q94">
+        <v>3.75</v>
+      </c>
+      <c r="R94">
+        <v>64.2</v>
+      </c>
+      <c r="S94">
+        <v>13463.778</v>
+      </c>
+      <c r="T94">
+        <v>33904.97637714286</v>
       </c>
     </row>
     <row r="95">
@@ -4717,10 +6137,25 @@
         <v>1.372038</v>
       </c>
       <c r="N95">
-        <v>458.75</v>
+        <v>334.63</v>
       </c>
       <c r="O95">
-        <v>334.63</v>
+        <v>5.12</v>
+      </c>
+      <c r="P95">
+        <v>4.83</v>
+      </c>
+      <c r="Q95">
+        <v>3.9</v>
+      </c>
+      <c r="R95">
+        <v>71.5</v>
+      </c>
+      <c r="S95">
+        <v>14033.091</v>
+      </c>
+      <c r="T95">
+        <v>34777.2001965</v>
       </c>
     </row>
     <row r="96">
@@ -4761,10 +6196,25 @@
         <v>1.424562</v>
       </c>
       <c r="N96">
-        <v>528.75</v>
+        <v>385.63</v>
       </c>
       <c r="O96">
-        <v>385.63</v>
+        <v>5.33</v>
+      </c>
+      <c r="P96">
+        <v>4.9</v>
+      </c>
+      <c r="Q96">
+        <v>4.17</v>
+      </c>
+      <c r="R96">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="S96">
+        <v>13739.497</v>
+      </c>
+      <c r="T96">
+        <v>34880.65659217391</v>
       </c>
     </row>
     <row r="97">
@@ -4805,10 +6255,25 @@
         <v>1.53748</v>
       </c>
       <c r="N97">
-        <v>527.9</v>
+        <v>380</v>
       </c>
       <c r="O97">
-        <v>380</v>
+        <v>5.33</v>
+      </c>
+      <c r="P97">
+        <v>5.02</v>
+      </c>
+      <c r="Q97">
+        <v>4.38</v>
+      </c>
+      <c r="R97">
+        <v>67.8</v>
+      </c>
+      <c r="S97">
+        <v>13585.842</v>
+      </c>
+      <c r="T97">
+        <v>34318.890821</v>
       </c>
     </row>
     <row r="98">
@@ -4849,10 +6314,25 @@
         <v>1.58395</v>
       </c>
       <c r="N98">
-        <v>534.75</v>
+        <v>411.38</v>
       </c>
       <c r="O98">
-        <v>411.38</v>
+        <v>5.33</v>
+      </c>
+      <c r="P98">
+        <v>5.07</v>
+      </c>
+      <c r="Q98">
+        <v>4.8</v>
+      </c>
+      <c r="R98">
+        <v>63.8</v>
+      </c>
+      <c r="S98">
+        <v>13199.428</v>
+      </c>
+      <c r="T98">
+        <v>33319.49272090909</v>
       </c>
     </row>
     <row r="99">
@@ -4893,10 +6373,25 @@
         <v>1.667497</v>
       </c>
       <c r="N99">
-        <v>535.63</v>
+        <v>385.5</v>
       </c>
       <c r="O99">
-        <v>385.5</v>
+        <v>5.33</v>
+      </c>
+      <c r="P99">
+        <v>4.88</v>
+      </c>
+      <c r="Q99">
+        <v>4.5</v>
+      </c>
+      <c r="R99">
+        <v>61.3</v>
+      </c>
+      <c r="S99">
+        <v>13913.16</v>
+      </c>
+      <c r="T99">
+        <v>34704.50241904762</v>
       </c>
     </row>
     <row r="100">
@@ -4937,10 +6432,25 @@
         <v>1.6336</v>
       </c>
       <c r="N100">
-        <v>563.75</v>
+        <v>354</v>
       </c>
       <c r="O100">
-        <v>354</v>
+        <v>5.33</v>
+      </c>
+      <c r="P100">
+        <v>4.46</v>
+      </c>
+      <c r="Q100">
+        <v>4.02</v>
+      </c>
+      <c r="R100">
+        <v>69.7</v>
+      </c>
+      <c r="S100">
+        <v>14690.493</v>
+      </c>
+      <c r="T100">
+        <v>36947.9275395</v>
       </c>
     </row>
     <row r="101">
@@ -4981,10 +6491,25 @@
         <v>1.56618</v>
       </c>
       <c r="N101">
-        <v>596.25</v>
+        <v>335.38</v>
       </c>
       <c r="O101">
-        <v>335.38</v>
+        <v>5.33</v>
+      </c>
+      <c r="P101">
+        <v>4.32</v>
+      </c>
+      <c r="Q101">
+        <v>4.06</v>
+      </c>
+      <c r="R101">
+        <v>79</v>
+      </c>
+      <c r="S101">
+        <v>15081.388</v>
+      </c>
+      <c r="T101">
+        <v>37763.9548</v>
       </c>
     </row>
     <row r="102">
@@ -5025,10 +6550,25 @@
         <v>1.51528</v>
       </c>
       <c r="N102">
-        <v>583.8099999999999</v>
+        <v>351.25</v>
       </c>
       <c r="O102">
-        <v>351.25</v>
+        <v>5.33</v>
+      </c>
+      <c r="P102">
+        <v>4.54</v>
+      </c>
+      <c r="Q102">
+        <v>4.21</v>
+      </c>
+      <c r="R102">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="S102">
+        <v>15808.935</v>
+      </c>
+      <c r="T102">
+        <v>38720.51797</v>
       </c>
     </row>
     <row r="103">
@@ -5069,10 +6609,25 @@
         <v>1.528088</v>
       </c>
       <c r="N103">
-        <v>617.5</v>
+        <v>330</v>
       </c>
       <c r="O103">
-        <v>330</v>
+        <v>5.33</v>
+      </c>
+      <c r="P103">
+        <v>4.59</v>
+      </c>
+      <c r="Q103">
+        <v>4.21</v>
+      </c>
+      <c r="R103">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="S103">
+        <v>16216.296</v>
+      </c>
+      <c r="T103">
+        <v>39105.5199235</v>
       </c>
     </row>
     <row r="104">
@@ -5113,10 +6668,25 @@
         <v>1.439838</v>
       </c>
       <c r="N104">
-        <v>545</v>
+        <v>320</v>
       </c>
       <c r="O104">
-        <v>320</v>
+        <v>5.33</v>
+      </c>
+      <c r="P104">
+        <v>4.87</v>
+      </c>
+      <c r="Q104">
+        <v>4.54</v>
+      </c>
+      <c r="R104">
+        <v>77.2</v>
+      </c>
+      <c r="S104">
+        <v>15950.864</v>
+      </c>
+      <c r="T104">
+        <v>38401.21733090909</v>
       </c>
     </row>
     <row r="105">
@@ -5157,10 +6727,25 @@
         <v>1.514766</v>
       </c>
       <c r="N105">
-        <v>522</v>
+        <v>284.8</v>
       </c>
       <c r="O105">
-        <v>284.8</v>
+        <v>5.33</v>
+      </c>
+      <c r="P105">
+        <v>4.86</v>
+      </c>
+      <c r="Q105">
+        <v>4.48</v>
+      </c>
+      <c r="R105">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="S105">
+        <v>16536.317</v>
+      </c>
+      <c r="T105">
+        <v>39129.39044772727</v>
       </c>
     </row>
     <row r="106">
@@ -5201,10 +6786,25 @@
         <v>1.400868</v>
       </c>
       <c r="N106">
-        <v>543</v>
+        <v>336.25</v>
       </c>
       <c r="O106">
-        <v>336.25</v>
+        <v>5.33</v>
+      </c>
+      <c r="P106">
+        <v>4.74</v>
+      </c>
+      <c r="Q106">
+        <v>4.31</v>
+      </c>
+      <c r="R106">
+        <v>68.2</v>
+      </c>
+      <c r="S106">
+        <v>17495.892</v>
+      </c>
+      <c r="T106">
+        <v>38903.73067578948</v>
       </c>
     </row>
     <row r="107">
@@ -5245,10 +6845,25 @@
         <v>1.33496</v>
       </c>
       <c r="N107">
-        <v>539.4</v>
+        <v>342.5</v>
       </c>
       <c r="O107">
-        <v>342.5</v>
+        <v>5.33</v>
+      </c>
+      <c r="P107">
+        <v>4.5</v>
+      </c>
+      <c r="Q107">
+        <v>4.25</v>
+      </c>
+      <c r="R107">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="S107">
+        <v>17963.291</v>
+      </c>
+      <c r="T107">
+        <v>40086.031605</v>
       </c>
     </row>
     <row r="108">
@@ -5289,10 +6904,25 @@
         <v>1.383168</v>
       </c>
       <c r="N108">
-        <v>546</v>
+        <v>342.5</v>
       </c>
       <c r="O108">
-        <v>342.5</v>
+        <v>5.33</v>
+      </c>
+      <c r="P108">
+        <v>3.97</v>
+      </c>
+      <c r="Q108">
+        <v>3.87</v>
+      </c>
+      <c r="R108">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="S108">
+        <v>17268.269</v>
+      </c>
+      <c r="T108">
+        <v>40310.81445409091</v>
       </c>
     </row>
     <row r="109">
@@ -5333,10 +6963,25 @@
         <v>1.453025</v>
       </c>
       <c r="N109">
-        <v>554.75</v>
+        <v>337.5</v>
       </c>
       <c r="O109">
-        <v>337.5</v>
+        <v>5.13</v>
+      </c>
+      <c r="P109">
+        <v>3.62</v>
+      </c>
+      <c r="Q109">
+        <v>3.72</v>
+      </c>
+      <c r="R109">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="S109">
+        <v>17599.23</v>
+      </c>
+      <c r="T109">
+        <v>41490.882814</v>
       </c>
     </row>
     <row r="110">
@@ -5377,10 +7022,25 @@
         <v>1.480128</v>
       </c>
       <c r="N110">
-        <v>573.4400000000001</v>
+        <v>374.75</v>
       </c>
       <c r="O110">
-        <v>374.75</v>
+        <v>4.83</v>
+      </c>
+      <c r="P110">
+        <v>3.97</v>
+      </c>
+      <c r="Q110">
+        <v>4.1</v>
+      </c>
+      <c r="R110">
+        <v>70.5</v>
+      </c>
+      <c r="S110">
+        <v>18316.116</v>
+      </c>
+      <c r="T110">
+        <v>42494.19735086957</v>
       </c>
     </row>
     <row r="111">
@@ -5421,10 +7081,25 @@
         <v>1.519686</v>
       </c>
       <c r="N111">
-        <v>574.5</v>
+        <v>352.3</v>
       </c>
       <c r="O111">
-        <v>352.3</v>
+        <v>4.64</v>
+      </c>
+      <c r="P111">
+        <v>4.26</v>
+      </c>
+      <c r="Q111">
+        <v>4.36</v>
+      </c>
+      <c r="R111">
+        <v>71.8</v>
+      </c>
+      <c r="S111">
+        <v>18961.4</v>
+      </c>
+      <c r="T111">
+        <v>43716.9269535</v>
       </c>
     </row>
     <row r="112">
@@ -5465,10 +7140,25 @@
         <v>1.417642</v>
       </c>
       <c r="N112">
-        <v>568.33</v>
+        <v>352</v>
       </c>
       <c r="O112">
-        <v>352</v>
+        <v>4.48</v>
+      </c>
+      <c r="P112">
+        <v>4.23</v>
+      </c>
+      <c r="Q112">
+        <v>4.39</v>
+      </c>
+      <c r="R112">
+        <v>74</v>
+      </c>
+      <c r="S112">
+        <v>19734.564</v>
+      </c>
+      <c r="T112">
+        <v>43655.57087047619</v>
       </c>
     </row>
     <row r="113">
@@ -5509,10 +7199,25 @@
         <v>1.544927</v>
       </c>
       <c r="N113">
-        <v>582.7</v>
+        <v>380.5</v>
       </c>
       <c r="O113">
-        <v>380.5</v>
+        <v>4.33</v>
+      </c>
+      <c r="P113">
+        <v>4.27</v>
+      </c>
+      <c r="Q113">
+        <v>4.63</v>
+      </c>
+      <c r="R113">
+        <v>71.7</v>
+      </c>
+      <c r="S113">
+        <v>19565.044</v>
+      </c>
+      <c r="T113">
+        <v>43524.3486335</v>
       </c>
     </row>
     <row r="114">
@@ -5553,10 +7258,25 @@
         <v>1.628226</v>
       </c>
       <c r="N114">
-        <v>603.75</v>
+        <v>436.5</v>
       </c>
       <c r="O114">
-        <v>436.5</v>
+        <v>4.33</v>
+      </c>
+      <c r="P114">
+        <v>4.21</v>
+      </c>
+      <c r="Q114">
+        <v>4.45</v>
+      </c>
+      <c r="R114">
+        <v>64.7</v>
+      </c>
+      <c r="S114">
+        <v>19547.281</v>
+      </c>
+      <c r="T114">
+        <v>44209.30962263158</v>
       </c>
     </row>
     <row r="115">
@@ -5597,10 +7317,25 @@
         <v>1.627835</v>
       </c>
       <c r="N115">
-        <v>615.13</v>
+        <v>394.5</v>
       </c>
       <c r="O115">
-        <v>394.5</v>
+        <v>4.33</v>
+      </c>
+      <c r="P115">
+        <v>3.97</v>
+      </c>
+      <c r="Q115">
+        <v>4.28</v>
+      </c>
+      <c r="R115">
+        <v>57</v>
+      </c>
+      <c r="S115">
+        <v>17828.026</v>
+      </c>
+      <c r="T115">
+        <v>42092.12872047619</v>
       </c>
     </row>
     <row r="116">
@@ -5641,10 +7376,25 @@
         <v>1.739932</v>
       </c>
       <c r="N116">
-        <v>635</v>
+        <v>386.88</v>
       </c>
       <c r="O116">
-        <v>386.88</v>
+        <v>4.33</v>
+      </c>
+      <c r="P116">
+        <v>3.78</v>
+      </c>
+      <c r="Q116">
+        <v>4.28</v>
+      </c>
+      <c r="R116">
+        <v>52.2</v>
+      </c>
+      <c r="S116">
+        <v>16678.46</v>
+      </c>
+      <c r="T116">
+        <v>39876.32775380952</v>
       </c>
     </row>
     <row r="117">
@@ -5685,10 +7435,25 @@
         <v>1.778867</v>
       </c>
       <c r="N117">
-        <v>669.2</v>
+        <v>392</v>
       </c>
       <c r="O117">
-        <v>392</v>
+        <v>4.33</v>
+      </c>
+      <c r="P117">
+        <v>3.92</v>
+      </c>
+      <c r="Q117">
+        <v>4.42</v>
+      </c>
+      <c r="R117">
+        <v>52.2</v>
+      </c>
+      <c r="S117">
+        <v>18642.368</v>
+      </c>
+      <c r="T117">
+        <v>41864.24535</v>
       </c>
     </row>
     <row r="118">
@@ -5729,10 +7494,25 @@
         <v>1.781535</v>
       </c>
       <c r="N118">
-        <v>715.38</v>
+        <v>420.5</v>
       </c>
       <c r="O118">
-        <v>420.5</v>
+        <v>4.33</v>
+      </c>
+      <c r="P118">
+        <v>3.89</v>
+      </c>
+      <c r="Q118">
+        <v>4.38</v>
+      </c>
+      <c r="R118">
+        <v>60.7</v>
+      </c>
+      <c r="S118">
+        <v>19673.301</v>
+      </c>
+      <c r="T118">
+        <v>42752.938085</v>
       </c>
     </row>
     <row r="119">
@@ -5773,10 +7553,25 @@
         <v>1.777264</v>
       </c>
       <c r="N119">
-        <v>736</v>
+        <v>496</v>
       </c>
       <c r="O119">
-        <v>496</v>
+        <v>4.33</v>
+      </c>
+      <c r="P119">
+        <v>3.88</v>
+      </c>
+      <c r="Q119">
+        <v>4.39</v>
+      </c>
+      <c r="R119">
+        <v>61.7</v>
+      </c>
+      <c r="S119">
+        <v>20784.895</v>
+      </c>
+      <c r="T119">
+        <v>44499.74130090909</v>
       </c>
     </row>
     <row r="120">
@@ -5817,10 +7612,25 @@
         <v>1.67167</v>
       </c>
       <c r="N120">
-        <v>795.1</v>
+        <v>507.7</v>
       </c>
       <c r="O120">
-        <v>507.7</v>
+        <v>4.33</v>
+      </c>
+      <c r="P120">
+        <v>3.7</v>
+      </c>
+      <c r="Q120">
+        <v>4.26</v>
+      </c>
+      <c r="R120">
+        <v>58.2</v>
+      </c>
+      <c r="S120">
+        <v>21383.587</v>
+      </c>
+      <c r="T120">
+        <v>44764.85063285715</v>
       </c>
     </row>
     <row r="121">
@@ -5861,10 +7671,25 @@
         <v>1.743768</v>
       </c>
       <c r="N121">
-        <v>780.63</v>
+        <v>461.13</v>
       </c>
       <c r="O121">
-        <v>461.13</v>
+        <v>4.22</v>
+      </c>
+      <c r="P121">
+        <v>3.57</v>
+      </c>
+      <c r="Q121">
+        <v>4.12</v>
+      </c>
+      <c r="R121">
+        <v>55.1</v>
+      </c>
+      <c r="S121">
+        <v>22188.588</v>
+      </c>
+      <c r="T121">
+        <v>45908.10230666667</v>
       </c>
     </row>
     <row r="122">
@@ -5905,10 +7730,25 @@
         <v>1.718656</v>
       </c>
       <c r="N122">
-        <v>754</v>
+        <v>394.4</v>
       </c>
       <c r="O122">
-        <v>394.4</v>
+        <v>4.09</v>
+      </c>
+      <c r="P122">
+        <v>3.52</v>
+      </c>
+      <c r="Q122">
+        <v>4.06</v>
+      </c>
+      <c r="R122">
+        <v>53.6</v>
+      </c>
+      <c r="S122">
+        <v>23003.126</v>
+      </c>
+      <c r="T122">
+        <v>46709.67221478261</v>
       </c>
     </row>
     <row r="123">
@@ -5949,10 +7789,25 @@
         <v>1.769985</v>
       </c>
       <c r="N123">
-        <v>708.25</v>
+        <v>409.25</v>
       </c>
       <c r="O123">
-        <v>409.25</v>
+        <v>3.88</v>
+      </c>
+      <c r="P123">
+        <v>3.55</v>
+      </c>
+      <c r="Q123">
+        <v>4.09</v>
+      </c>
+      <c r="R123">
+        <v>51</v>
+      </c>
+      <c r="S123">
+        <v>23023.623</v>
+      </c>
+      <c r="T123">
+        <v>47016.37417789474</v>
       </c>
     </row>
     <row r="124">
@@ -5993,10 +7848,25 @@
         <v>1.780704</v>
       </c>
       <c r="N124">
-        <v>627.5</v>
+        <v>392.5</v>
       </c>
       <c r="O124">
-        <v>392.5</v>
+        <v>3.72</v>
+      </c>
+      <c r="P124">
+        <v>3.5</v>
+      </c>
+      <c r="Q124">
+        <v>4.14</v>
+      </c>
+      <c r="R124">
+        <v>52.9</v>
+      </c>
+      <c r="S124">
+        <v>23377.327</v>
+      </c>
+      <c r="T124">
+        <v>48118.86665545455</v>
       </c>
     </row>
     <row r="125">
@@ -6037,10 +7907,25 @@
         <v>1.746556</v>
       </c>
       <c r="N125">
-        <v>619.2</v>
+        <v>415.4</v>
       </c>
       <c r="O125">
-        <v>415.4</v>
+        <v>3.64</v>
+      </c>
+      <c r="P125">
+        <v>3.54</v>
+      </c>
+      <c r="Q125">
+        <v>4.21</v>
+      </c>
+      <c r="R125">
+        <v>56.4</v>
+      </c>
+      <c r="S125">
+        <v>23520.722</v>
+      </c>
+      <c r="T125">
+        <v>49138.2736345</v>
       </c>
     </row>
     <row r="126">
@@ -6081,10 +7966,25 @@
         <v>1.793168</v>
       </c>
       <c r="N126">
-        <v>626.5</v>
+        <v>472</v>
       </c>
       <c r="O126">
-        <v>472</v>
+        <v>3.64</v>
+      </c>
+      <c r="P126">
+        <v>3.47</v>
+      </c>
+      <c r="Q126">
+        <v>4.13</v>
+      </c>
+      <c r="R126">
+        <v>56.6</v>
+      </c>
+      <c r="S126">
+        <v>22892.923</v>
+      </c>
+      <c r="T126">
+        <v>49511.97204105263</v>
       </c>
     </row>
     <row r="127">
@@ -6125,10 +8025,25 @@
         <v>1.657704</v>
       </c>
       <c r="N127">
-        <v>658.25</v>
+        <v>725.63</v>
       </c>
       <c r="O127">
-        <v>725.63</v>
+        <v>3.64</v>
+      </c>
+      <c r="P127">
+        <v>3.71</v>
+      </c>
+      <c r="Q127">
+        <v>4.25</v>
+      </c>
+      <c r="R127">
+        <v>53.3</v>
+      </c>
+      <c r="S127">
+        <v>22130.038</v>
+      </c>
+      <c r="T127">
+        <v>46859.67223090909</v>
       </c>
     </row>
   </sheetData>

</xml_diff>